<commit_message>
Hoàn thiện hồ sơ nộp bài: bỏ mã nội bộ trong slide, sửa tham chiếu ngoài gói, thống nhất số liệu kiểm thử, đặt tác giả
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/tai_lieu_nop_bai/bang_chung_kiem_thu/3-Phieu-ket-qua-202-test-case.xlsx
+++ b/docs/tai_lieu_nop_bai/bang_chung_kiem_thu/3-Phieu-ket-qua-202-test-case.xlsx
@@ -14184,7 +14184,7 @@
       </c>
       <c r="H188" s="2" t="inlineStr">
         <is>
-          <t>Phục hồi thử vào CSDL tạm, số bản ghi chính khớp; CSDL đang chạy không bị đụng; CSDL tạm bị dọn.</t>
+          <t>Phục hồi thử vào CSDL tạm, số bản ghi chính khớp; CSDL đang chạy không bị tác động; CSDL tạm bị dọn.</t>
         </is>
       </c>
       <c r="I188" s="2" t="inlineStr">
@@ -16401,7 +16401,6 @@
         <v/>
       </c>
     </row>
-    <row r="31"/>
     <row r="32">
       <c r="A32" s="6" t="inlineStr">
         <is>
@@ -19404,7 +19403,7 @@
       </c>
       <c r="C130" s="7" t="inlineStr">
         <is>
-          <t>`backup:verify` phục hồi thử vào CSDL tạm và xác nhận số bản ghi chính khớp bản gốc, không đụng CSDL đang chạy.</t>
+          <t>`backup:verify` phục hồi thử vào CSDL tạm và xác nhận số bản ghi chính khớp bản gốc, không can thiệp CSDL đang chạy.</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">

</xml_diff>